<commit_message>
Added to the train set
</commit_message>
<xml_diff>
--- a/datasets/train.xlsx
+++ b/datasets/train.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ssvzwng\Desktop\tuouvous\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5ADF4676-9AAB-4D37-BF3A-B1C34B85C37B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E0B07F7-2DB0-4068-866D-155E65D5FF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F95B6576-85E5-4B51-9FB5-90017593C264}"/>
   </bookViews>
@@ -31,6 +31,161 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="50">
+  <si>
+    <t>register</t>
+  </si>
+  <si>
+    <t>english</t>
+  </si>
+  <si>
+    <t>french</t>
+  </si>
+  <si>
+    <t>Je t'kiffe.</t>
+  </si>
+  <si>
+    <t>Je tiens énormément à toi.</t>
+  </si>
+  <si>
+    <t>Je t'aime.</t>
+  </si>
+  <si>
+    <t>Je vous aime profondément.</t>
+  </si>
+  <si>
+    <t>Veuillez recevoir l'expression de mon profond attachement.</t>
+  </si>
+  <si>
+    <t>I love you.</t>
+  </si>
+  <si>
+    <t>STREET</t>
+  </si>
+  <si>
+    <t>CONVERSATIONAL</t>
+  </si>
+  <si>
+    <t>STANDARD</t>
+  </si>
+  <si>
+    <t>FORMAL</t>
+  </si>
+  <si>
+    <t>ADMINISTRATIVE</t>
+  </si>
+  <si>
+    <t>Do you have any suggestions ?</t>
+  </si>
+  <si>
+    <t>T'as des idées ?</t>
+  </si>
+  <si>
+    <t>Tu aurais une suggestion ?</t>
+  </si>
+  <si>
+    <t>As-tu des suggestions ?</t>
+  </si>
+  <si>
+    <t>Auriez-vous des suggestions ?</t>
+  </si>
+  <si>
+    <t>Auriez-vous des recommandations à formuler ?</t>
+  </si>
+  <si>
+    <t>You weren't supposed to know.</t>
+  </si>
+  <si>
+    <t>Tu n'étais pas censé le savoir.</t>
+  </si>
+  <si>
+    <t>Vous n'étiez pas censé le savoir.</t>
+  </si>
+  <si>
+    <t>Vous n'étiez pas censé avoir connaissance de cette information.</t>
+  </si>
+  <si>
+    <t>T'étais pas censé capter ça.</t>
+  </si>
+  <si>
+    <t>Tu n'aurais jamais dû apprendre ça.</t>
+  </si>
+  <si>
+    <t>That's not gonna work.</t>
+  </si>
+  <si>
+    <t>Ça va pas le faire.</t>
+  </si>
+  <si>
+    <t>Ça marchera pas.</t>
+  </si>
+  <si>
+    <t>Ça ne marchera pas.</t>
+  </si>
+  <si>
+    <t>Cela ne fonctionnera pas.</t>
+  </si>
+  <si>
+    <t>Cette solution n'est pas envisageable.</t>
+  </si>
+  <si>
+    <t>I need some help.</t>
+  </si>
+  <si>
+    <t>J'ai besoin d'un coup de main.</t>
+  </si>
+  <si>
+    <t>J'ai besoin d'un peu d'aide.</t>
+  </si>
+  <si>
+    <t>J'ai besoin d'aide.</t>
+  </si>
+  <si>
+    <t>J'aurais besoin de votre aide.</t>
+  </si>
+  <si>
+    <t>Je requiers une assistance.</t>
+  </si>
+  <si>
+    <t>Ça fait un bail.</t>
+  </si>
+  <si>
+    <t>Ça fait un moment.</t>
+  </si>
+  <si>
+    <t>Ça fait longtemps.</t>
+  </si>
+  <si>
+    <t>Une longue période s'est écoulée depuis notre dernier échange.</t>
+  </si>
+  <si>
+    <t>Cela fait longtemps que nous ne nous sommes pas vus.</t>
+  </si>
+  <si>
+    <t>It's been a long time.</t>
+  </si>
+  <si>
+    <t>I can't believe he did that.</t>
+  </si>
+  <si>
+    <t>Je bugue grave qu'il ait fait ça.</t>
+  </si>
+  <si>
+    <t>Il est difficile de croire qu'il ait agi de cette manière.</t>
+  </si>
+  <si>
+    <t>Je suis stupéfait qu'il ait fait cela.</t>
+  </si>
+  <si>
+    <t>Je n'arrive pas à croire qu'il ait fait ça.</t>
+  </si>
+  <si>
+    <t>J'en reviens pas qu'il ait fait ça.</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -380,9 +535,411 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{903655B4-DA13-47A5-888D-532BF9DF7DF6}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="18.7265625" customWidth="1"/>
+    <col min="2" max="2" width="29.81640625" customWidth="1"/>
+    <col min="3" max="3" width="55.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C32" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>12</v>
+      </c>
+      <c r="B35" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" t="s">
+        <v>44</v>
+      </c>
+      <c r="C36" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added more to the train set
</commit_message>
<xml_diff>
--- a/datasets/train.xlsx
+++ b/datasets/train.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ssvzwng\Desktop\tuouvous\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E0B07F7-2DB0-4068-866D-155E65D5FF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D98F229-3BEE-4FF7-9C15-8EA461696008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F95B6576-85E5-4B51-9FB5-90017593C264}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="92">
   <si>
     <t>register</t>
   </si>
@@ -184,6 +184,132 @@
   </si>
   <si>
     <t>J'en reviens pas qu'il ait fait ça.</t>
+  </si>
+  <si>
+    <t>Shut up.</t>
+  </si>
+  <si>
+    <t>Ta gueule.</t>
+  </si>
+  <si>
+    <t>La ferme.</t>
+  </si>
+  <si>
+    <t>Tais-toi.</t>
+  </si>
+  <si>
+    <t>Veuillez vous taire.</t>
+  </si>
+  <si>
+    <t>Je vous prie de bien vouloir garder le silence.</t>
+  </si>
+  <si>
+    <t>Au nom de quoi vous permettez-vous d'agir ainsi ?</t>
+  </si>
+  <si>
+    <t>Mais t'es qui, toi ?</t>
+  </si>
+  <si>
+    <t>Pour qui vous prenez-vous ?</t>
+  </si>
+  <si>
+    <t>Pour qui tu te prends ?</t>
+  </si>
+  <si>
+    <t>Pour qui te prends-tu ?</t>
+  </si>
+  <si>
+    <t>Who do you think you are ?</t>
+  </si>
+  <si>
+    <t>I agree.</t>
+  </si>
+  <si>
+    <t>Je partage votre avis.</t>
+  </si>
+  <si>
+    <t>J'exprime mon accord.</t>
+  </si>
+  <si>
+    <t>Je suis d'accord.</t>
+  </si>
+  <si>
+    <t>Tout à fait d'accord.</t>
+  </si>
+  <si>
+    <t>Grave.</t>
+  </si>
+  <si>
+    <t>Avez-vous eu l'occasion de vous rendre au restaurant que je vous avais recommandé ?</t>
+  </si>
+  <si>
+    <t>Êtes-vous allé au restaurant dont je vous ai parlé ?</t>
+  </si>
+  <si>
+    <t>Tu es allé au restaurant dont je t'ai parlé ?</t>
+  </si>
+  <si>
+    <t>Alors, t'es allé au resto dont je t'ai parlé ?</t>
+  </si>
+  <si>
+    <t>Du coup, t'as testé le resto ?</t>
+  </si>
+  <si>
+    <t>Did you go to the restaurant I told you about ?</t>
+  </si>
+  <si>
+    <t>Comment avez-vous pu nous infliger une telle situation ?</t>
+  </si>
+  <si>
+    <t>Comment avez-vous pu nous faire cela ?</t>
+  </si>
+  <si>
+    <t>Comment as-tu pu nous faire ça ?</t>
+  </si>
+  <si>
+    <t>Comment t'as pu nous faire ça ?</t>
+  </si>
+  <si>
+    <t>How could you do this to us?</t>
+  </si>
+  <si>
+    <t>Comment t'as pu nous la faire à l'envers ?</t>
+  </si>
+  <si>
+    <t>You did not meet our standards.</t>
+  </si>
+  <si>
+    <t>Vous n'avez pas satisfait à nos exigences.</t>
+  </si>
+  <si>
+    <t>T'étais pas à la hauteur.</t>
+  </si>
+  <si>
+    <t>Vous n'avez pas répondu à nos attentes.</t>
+  </si>
+  <si>
+    <t>Vous ne correspondez pas aux standards attendus.</t>
+  </si>
+  <si>
+    <t>T'as pas le niveau.</t>
+  </si>
+  <si>
+    <t>What do you mean ?</t>
+  </si>
+  <si>
+    <t>Pourriez-vous préciser le sens de votre propos ?</t>
+  </si>
+  <si>
+    <t>Qu'est-ce que vous voulez dire ?</t>
+  </si>
+  <si>
+    <t>Qu'est-ce que tu veux dire ?</t>
+  </si>
+  <si>
+    <t>Tu racontes quoi, là ?</t>
+  </si>
+  <si>
+    <t>Que souhaitez-vous dire exactement ?</t>
   </si>
 </sst>
 </file>
@@ -535,12 +661,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{903655B4-DA13-47A5-888D-532BF9DF7DF6}">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.7265625" customWidth="1"/>
-    <col min="2" max="2" width="29.81640625" customWidth="1"/>
-    <col min="3" max="3" width="55.90625" customWidth="1"/>
+    <col min="2" max="2" width="41.7265625" customWidth="1"/>
+    <col min="3" max="3" width="77.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -939,6 +1065,391 @@
         <v>46</v>
       </c>
     </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38" t="s">
+        <v>50</v>
+      </c>
+      <c r="C38" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" t="s">
+        <v>50</v>
+      </c>
+      <c r="C39" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" t="s">
+        <v>50</v>
+      </c>
+      <c r="C40" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42" t="s">
+        <v>61</v>
+      </c>
+      <c r="C42" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>10</v>
+      </c>
+      <c r="B43" t="s">
+        <v>61</v>
+      </c>
+      <c r="C43" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>11</v>
+      </c>
+      <c r="B44" t="s">
+        <v>61</v>
+      </c>
+      <c r="C44" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" t="s">
+        <v>61</v>
+      </c>
+      <c r="C45" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>13</v>
+      </c>
+      <c r="B46" t="s">
+        <v>61</v>
+      </c>
+      <c r="C46" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" t="s">
+        <v>62</v>
+      </c>
+      <c r="C47" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>10</v>
+      </c>
+      <c r="B48" t="s">
+        <v>62</v>
+      </c>
+      <c r="C48" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>11</v>
+      </c>
+      <c r="B49" t="s">
+        <v>62</v>
+      </c>
+      <c r="C49" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>12</v>
+      </c>
+      <c r="B50" t="s">
+        <v>62</v>
+      </c>
+      <c r="C50" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>13</v>
+      </c>
+      <c r="B51" t="s">
+        <v>62</v>
+      </c>
+      <c r="C51" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>9</v>
+      </c>
+      <c r="B52" t="s">
+        <v>73</v>
+      </c>
+      <c r="C52" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>10</v>
+      </c>
+      <c r="B53" t="s">
+        <v>73</v>
+      </c>
+      <c r="C53" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>11</v>
+      </c>
+      <c r="B54" t="s">
+        <v>73</v>
+      </c>
+      <c r="C54" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" t="s">
+        <v>73</v>
+      </c>
+      <c r="C55" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>13</v>
+      </c>
+      <c r="B56" t="s">
+        <v>73</v>
+      </c>
+      <c r="C56" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>9</v>
+      </c>
+      <c r="B57" t="s">
+        <v>78</v>
+      </c>
+      <c r="C57" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>10</v>
+      </c>
+      <c r="B58" t="s">
+        <v>78</v>
+      </c>
+      <c r="C58" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>11</v>
+      </c>
+      <c r="B59" t="s">
+        <v>78</v>
+      </c>
+      <c r="C59" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>12</v>
+      </c>
+      <c r="B60" t="s">
+        <v>78</v>
+      </c>
+      <c r="C60" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>13</v>
+      </c>
+      <c r="B61" t="s">
+        <v>78</v>
+      </c>
+      <c r="C61" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>9</v>
+      </c>
+      <c r="B62" t="s">
+        <v>80</v>
+      </c>
+      <c r="C62" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>10</v>
+      </c>
+      <c r="B63" t="s">
+        <v>80</v>
+      </c>
+      <c r="C63" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>11</v>
+      </c>
+      <c r="B64" t="s">
+        <v>80</v>
+      </c>
+      <c r="C64" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>12</v>
+      </c>
+      <c r="B65" t="s">
+        <v>80</v>
+      </c>
+      <c r="C65" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>13</v>
+      </c>
+      <c r="B66" t="s">
+        <v>80</v>
+      </c>
+      <c r="C66" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>9</v>
+      </c>
+      <c r="B67" t="s">
+        <v>86</v>
+      </c>
+      <c r="C67" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>10</v>
+      </c>
+      <c r="B68" t="s">
+        <v>86</v>
+      </c>
+      <c r="C68" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>11</v>
+      </c>
+      <c r="B69" t="s">
+        <v>86</v>
+      </c>
+      <c r="C69" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>12</v>
+      </c>
+      <c r="B70" t="s">
+        <v>86</v>
+      </c>
+      <c r="C70" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>13</v>
+      </c>
+      <c r="B71" t="s">
+        <v>86</v>
+      </c>
+      <c r="C71" t="s">
+        <v>87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>